<commit_message>
fix error caused by incorrectly trying to parse condition format text as a formula
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/ConditionalFormatting/CFContains.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/ConditionalFormatting/CFContains.xlsx
@@ -16,16 +16,19 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:si>
-    <x:t>Hello</x:t>
+    <x:t>Number 5</x:t>
   </x:si>
   <x:si>
-    <x:t>Hellos</x:t>
+    <x:t>The Number 5</x:t>
   </x:si>
   <x:si>
-    <x:t>Hell</x:t>
+    <x:t>Number 50</x:t>
   </x:si>
   <x:si>
-    <x:t>Holl</x:t>
+    <x:t>Number 4</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Nomber 5</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -90,7 +93,7 @@
       <x:fill>
         <x:patternFill patternType="solid">
           <x:fgColor auto="1"/>
-          <x:bgColor rgb="FFFF0000"/>
+          <x:bgColor rgb="FFFFFF00"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -386,7 +389,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:A4"/>
+  <x:dimension ref="A1:A5"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:1">
@@ -409,10 +412,15 @@
         <x:v>3</x:v>
       </x:c>
     </x:row>
+    <x:row r="5" spans="1:1">
+      <x:c r="A5" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="A1:A4">
-    <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Hell">
-      <x:formula>NOT(ISERROR(SEARCH("Hell",A1)))</x:formula>
+  <x:conditionalFormatting sqref="A1:A5">
+    <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Number 5">
+      <x:formula>NOT(ISERROR(SEARCH("Number 5",A1)))</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>

</xml_diff>